<commit_message>
refactor(controllers): streamline query parameters and enhance UI consistency
- Removed unused status filters from ProcurementPurchaseOrderController and ProcurementReceiptController to simplify query handling.
- Updated UserController to improve status filtering logic, ensuring clearer handling of active and inactive user states.
- Enhanced dashboard view styles for better visual consistency across various statistics.
- Improved error handling and user feedback in forms and modals, ensuring a more intuitive user experience.
- Refactored asset management views to enhance clarity and maintainability, including updates to asset detail and document management interfaces.
</commit_message>
<xml_diff>
--- a/public/docs/ImportVendorTemplate.xlsx
+++ b/public/docs/ImportVendorTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ahwal\Documents\Template Exel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ACER\Documents\Collage\magang\asset_monitoring_web\public\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ACF5021-43D2-462D-B345-08EB2B26E370}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8E37412-DAAE-4AD2-8348-98197250DB17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="60" windowWidth="20400" windowHeight="11835" xr2:uid="{B84E10DA-0A94-4A2A-9F95-204D239DF1FA}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="9420" xr2:uid="{B84E10DA-0A94-4A2A-9F95-204D239DF1FA}"/>
   </bookViews>
   <sheets>
     <sheet name="Import Vendor" sheetId="1" r:id="rId1"/>
@@ -73,9 +73,6 @@
     <t>supplie@supplied.com</t>
   </si>
   <si>
-    <t>Nama Vedor</t>
-  </si>
-  <si>
     <t>Kontak Person</t>
   </si>
   <si>
@@ -104,6 +101,9 @@
   </si>
   <si>
     <t>NOTE :BUKA BATAS PENGISIAN</t>
+  </si>
+  <si>
+    <t>Nama Vendor</t>
   </si>
 </sst>
 </file>
@@ -242,7 +242,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -268,19 +268,15 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -598,39 +594,39 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E17F584E-BF30-4BA1-A8DD-D2A5DE90FCC4}">
   <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
-    <col min="2" max="2" width="15.140625" customWidth="1"/>
-    <col min="3" max="3" width="17.7109375" customWidth="1"/>
-    <col min="4" max="4" width="23.140625" customWidth="1"/>
+    <col min="2" max="2" width="15.109375" customWidth="1"/>
+    <col min="3" max="3" width="17.6640625" customWidth="1"/>
+    <col min="4" max="4" width="23.109375" customWidth="1"/>
     <col min="5" max="5" width="26" customWidth="1"/>
-    <col min="6" max="6" width="24.28515625" customWidth="1"/>
-    <col min="7" max="7" width="42.7109375" customWidth="1"/>
+    <col min="6" max="6" width="24.33203125" customWidth="1"/>
+    <col min="7" max="7" width="42.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="C1" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="D1" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="E1" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="F1" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="9" t="s">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="11" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="8" t="s">
@@ -639,17 +635,17 @@
       <c r="C2" s="8">
         <v>89737373</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="12" t="s">
         <v>3</v>
       </c>
       <c r="F2" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="16" t="s">
-        <v>22</v>
+      <c r="G2" s="13" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -667,24 +663,24 @@
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
   <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="16.5703125" customWidth="1"/>
-    <col min="3" max="3" width="28.7109375" customWidth="1"/>
-    <col min="4" max="4" width="31.7109375" customWidth="1"/>
-    <col min="5" max="5" width="60.140625" customWidth="1"/>
+    <col min="2" max="2" width="16.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.6640625" customWidth="1"/>
+    <col min="4" max="4" width="31.6640625" customWidth="1"/>
+    <col min="5" max="5" width="60.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="23.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="B1" s="15"/>
+    <row r="1" spans="1:5" ht="22.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="14"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="2"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
         <v>5</v>
@@ -699,7 +695,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="6"/>
       <c r="B3" s="7" t="s">
         <v>9</v>
@@ -711,13 +707,13 @@
         <v>10</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="6"/>
       <c r="B4" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C4" s="8">
         <v>100</v>
@@ -727,10 +723,10 @@
       </c>
       <c r="E4" s="9"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="6"/>
       <c r="B5" s="9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C5" s="8">
         <v>20</v>
@@ -740,10 +736,10 @@
       </c>
       <c r="E5" s="9"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="6"/>
       <c r="B6" s="9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C6" s="8">
         <v>100</v>
@@ -753,10 +749,10 @@
       </c>
       <c r="E6" s="9"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="6"/>
       <c r="B7" s="9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C7" s="8">
         <v>255</v>
@@ -766,10 +762,10 @@
       </c>
       <c r="E7" s="9"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="6"/>
-      <c r="B8" s="11" t="s">
-        <v>17</v>
+      <c r="B8" s="9" t="s">
+        <v>16</v>
       </c>
       <c r="C8" s="9"/>
       <c r="D8" s="8" t="s">

</xml_diff>